<commit_message>
feat: Acesso ao banco de dados
- UsersController.py (primeira consulta)
</commit_message>
<xml_diff>
--- a/api/desempenho/2025-07-01.xlsx
+++ b/api/desempenho/2025-07-01.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,18 +456,23 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>15:59:49</t>
+          <t>17:04:22</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>51238</v>
+        <v>57381</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
       </c>
       <c r="E2" t="n">
-        <v>54.6953125</v>
+        <v>79.33</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Usuário 127.0.0.1 acessou a rota Home</t>
+          <t>Usuário acessou a rota Home</t>
         </is>
       </c>
     </row>
@@ -479,11 +484,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>16:02:19</t>
+          <t>17:04:57</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>51490</v>
+        <v>57441</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -491,67 +496,11 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>54.43359375</v>
+        <v>78.91</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Usuário acessou a rota Home</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-07-01</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>16:02:32</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>51490</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>127.0.0.1</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>54.68359375</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Usuário acessou a rota Home</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025-07-01</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>16:02:33</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>51490</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>127.0.0.1</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>54.80859375</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Usuário acessou a rota Home</t>
+          <t>Usuário acessou a rota Users</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Resgatando dados (perfil dos Mentores - VIEW)
- UsersController.py (primeira consulta)
</commit_message>
<xml_diff>
--- a/api/desempenho/2025-07-01.xlsx
+++ b/api/desempenho/2025-07-01.xlsx
@@ -456,11 +456,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>17:04:22</t>
+          <t>17:21:11</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>57381</v>
+        <v>58875</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -468,11 +468,11 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>79.33</v>
+        <v>79.39</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Usuário acessou a rota Home</t>
+          <t>Usuário acessou a rota Users-Mentores (VIEW)</t>
         </is>
       </c>
     </row>
@@ -484,11 +484,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>17:04:57</t>
+          <t>17:21:13</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>57441</v>
+        <v>58875</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -496,11 +496,11 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>78.91</v>
+        <v>83.09</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Usuário acessou a rota Users</t>
+          <t>Usuário acessou a rota Users-Mentores (VIEW)</t>
         </is>
       </c>
     </row>

</xml_diff>